<commit_message>
feat: sync question bank, templates, and H5 review explanations
</commit_message>
<xml_diff>
--- a/frontend/public/templates/question-import-template.xlsx
+++ b/frontend/public/templates/question-import-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Questions" sheetId="1" r:id="rId1"/>
+    <sheet name="题目导入模板" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,107 +397,143 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>title</v>
+        <v>题目标题</v>
       </c>
       <c r="B1" t="str">
-        <v>content</v>
+        <v>题目内容</v>
       </c>
       <c r="C1" t="str">
-        <v>optionA</v>
+        <v>选项A</v>
       </c>
       <c r="D1" t="str">
-        <v>optionB</v>
+        <v>选项B</v>
       </c>
       <c r="E1" t="str">
-        <v>optionC</v>
+        <v>选项C</v>
       </c>
       <c r="F1" t="str">
-        <v>optionD</v>
+        <v>选项D</v>
       </c>
       <c r="G1" t="str">
-        <v>correctAnswer</v>
+        <v>选项E</v>
       </c>
       <c r="H1" t="str">
-        <v>difficulty</v>
+        <v>选项F</v>
       </c>
       <c r="I1" t="str">
-        <v>category</v>
+        <v>正确答案</v>
       </c>
       <c r="J1" t="str">
-        <v>points</v>
+        <v>题目难度</v>
+      </c>
+      <c r="K1" t="str">
+        <v>题目分类</v>
+      </c>
+      <c r="L1" t="str">
+        <v>分值</v>
+      </c>
+      <c r="M1" t="str">
+        <v>正确答案解析</v>
+      </c>
+      <c r="N1" t="str">
+        <v>错误答案解析</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>凯撒密码基础题</v>
+        <v>示例题目1</v>
       </c>
       <c r="B2" t="str">
-        <v>凯撒密码属于哪种加密方式？</v>
+        <v>《中华人民共和国密码法》自何时起施行？</v>
       </c>
       <c r="C2" t="str">
-        <v>替换加密</v>
+        <v>2019年10月26日</v>
       </c>
       <c r="D2" t="str">
-        <v>置换加密</v>
+        <v>2020年1月1日</v>
       </c>
       <c r="E2" t="str">
-        <v>哈希算法</v>
+        <v>2021年7月1日</v>
       </c>
       <c r="F2" t="str">
-        <v>分组加密</v>
+        <v>2020年6月1日</v>
       </c>
       <c r="G2" t="str">
-        <v>A</v>
+        <v/>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>B</v>
+      </c>
+      <c r="J2" t="str">
         <v>easy</v>
       </c>
-      <c r="I2" t="str">
-        <v>古典密码</v>
-      </c>
-      <c r="J2">
+      <c r="K2" t="str">
+        <v>密码安全</v>
+      </c>
+      <c r="L2">
         <v>5</v>
+      </c>
+      <c r="M2" t="str">
+        <v>《中华人民共和国密码法》自2020年1月1日起正式施行。</v>
+      </c>
+      <c r="N2" t="str">
+        <v>如果选错，重点回顾《密码法》的正式施行时间是2020年1月1日。</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>RSA题</v>
+        <v>示例题目2</v>
       </c>
       <c r="B3" t="str">
-        <v>RSA常见安全基础依赖于什么问题？</v>
+        <v>以下哪种做法有利于保护自己的密码安全？</v>
       </c>
       <c r="C3" t="str">
-        <v>离散对数</v>
+        <v>把密码写在便签纸上贴在电脑旁</v>
       </c>
       <c r="D3" t="str">
-        <v>大整数分解</v>
+        <v>所有平台使用同一个密码</v>
       </c>
       <c r="E3" t="str">
-        <v>哈希碰撞</v>
+        <v>定期更换密码并避免重复使用</v>
       </c>
       <c r="F3" t="str">
-        <v>最短路径</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
+        <v>使用连续数字如123456作为密码</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>medium</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>公钥密码</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
+        <v>C</v>
+      </c>
+      <c r="J3" t="str">
+        <v>easy</v>
+      </c>
+      <c r="K3" t="str">
+        <v>密码安全</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
+      <c r="M3" t="str">
+        <v>定期更换并避免重复使用密码，可以降低账号连带泄露风险。</v>
+      </c>
+      <c r="N3" t="str">
+        <v>如果答错，说明还需要强化“不要重复使用密码、不要使用弱密码”的安全意识。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>